<commit_message>
feat: write compensation amount in words to PRAE
</commit_message>
<xml_diff>
--- a/resources/Pauschale_Reiseaufwandsentschaedigung.xlsx
+++ b/resources/Pauschale_Reiseaufwandsentschaedigung.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="130">
   <si>
     <t xml:space="preserve">Aufzeichnung über Einsätze und Bestätigung über den Erhalt von
 pauschalen Reiseaufwandsentschädigungen</t>
@@ -41,9 +41,15 @@
     <t xml:space="preserve">Sozialversicherungsnummer:</t>
   </si>
   <si>
+    <t xml:space="preserve">{d.svn}</t>
+  </si>
+  <si>
     <t xml:space="preserve">Geburtsdatum:</t>
   </si>
   <si>
+    <t xml:space="preserve">{d.birthDate:formatD('DDMMYY')}</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ausländische Sozialversicherungsnummer*:</t>
   </si>
   <si>
@@ -51,6 +57,9 @@
   </si>
   <si>
     <t xml:space="preserve">Wohnanschrift:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{d.address}</t>
   </si>
   <si>
     <r>
@@ -507,6 +516,9 @@
     <t xml:space="preserve">in Worten:</t>
   </si>
   <si>
+    <t xml:space="preserve">{d.totalWords}</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="8"/>
@@ -990,6 +1002,9 @@
     <t xml:space="preserve">IBAN:</t>
   </si>
   <si>
+    <t xml:space="preserve">{d.iban}</t>
+  </si>
+  <si>
     <t xml:space="preserve">BIC:</t>
   </si>
   <si>
@@ -1035,6 +1050,9 @@
   </si>
   <si>
     <t xml:space="preserve">Der / Die angeführte(n) Einsatztag(e) stimmen mit den von uns geführten Aufzeichnungen überein und es wurden vom Verein / Verband keine zusätzlichen Aufwandsentschädigungen im oben angeführten Monat ausbezahlt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{d.generationDate}</t>
   </si>
   <si>
     <t xml:space="preserve">Verbandsstempel u. Unterschrift Vereins-/Verbands- Verantwortliche/r</t>
@@ -2181,7 +2199,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProps13.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" autoLine="false" print="true" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" autoLine="false" print="true" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProps14.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2193,11 +2211,11 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProps16.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" autoLine="false" print="true" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" autoLine="false" print="true" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProps17.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" autoLine="false" print="true" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" autoLine="false" print="true" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2225,7 +2243,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProps8.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" autoLine="false" print="true" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" autoLine="false" print="true" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProps9.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2243,9 +2261,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>30</xdr:col>
-      <xdr:colOff>111240</xdr:colOff>
+      <xdr:colOff>110160</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>106200</xdr:rowOff>
+      <xdr:rowOff>105120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2259,7 +2277,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="7960320" y="185400"/>
-          <a:ext cx="2834280" cy="378000"/>
+          <a:ext cx="2833200" cy="376920"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -3333,17 +3351,21 @@
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
-      <c r="D5" s="12"/>
+      <c r="D5" s="12" t="s">
+        <v>6</v>
+      </c>
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
       <c r="H5" s="13" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I5" s="13"/>
       <c r="J5" s="13"/>
       <c r="K5" s="13"/>
-      <c r="L5" s="14"/>
+      <c r="L5" s="14" t="s">
+        <v>8</v>
+      </c>
       <c r="M5" s="14"/>
       <c r="N5" s="14"/>
       <c r="O5" s="14"/>
@@ -3366,7 +3388,7 @@
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B6" s="16"/>
       <c r="C6" s="16"/>
@@ -3383,7 +3405,7 @@
       <c r="N6" s="17"/>
       <c r="O6" s="17"/>
       <c r="P6" s="18" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q6" s="18"/>
       <c r="R6" s="18"/>
@@ -3403,11 +3425,13 @@
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B7" s="19"/>
       <c r="C7" s="19"/>
-      <c r="D7" s="20"/>
+      <c r="D7" s="20" t="s">
+        <v>12</v>
+      </c>
       <c r="E7" s="20"/>
       <c r="F7" s="20"/>
       <c r="G7" s="20"/>
@@ -3438,7 +3462,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="21"/>
@@ -3473,10 +3497,10 @@
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C9" s="23"/>
       <c r="D9" s="23"/>
@@ -3484,7 +3508,7 @@
       <c r="F9" s="23"/>
       <c r="G9" s="23"/>
       <c r="H9" s="23" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="I9" s="23"/>
       <c r="J9" s="23"/>
@@ -3494,7 +3518,7 @@
       <c r="N9" s="23"/>
       <c r="O9" s="23"/>
       <c r="P9" s="23" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="Q9" s="23"/>
       <c r="R9" s="23"/>
@@ -3504,7 +3528,7 @@
       <c r="V9" s="23"/>
       <c r="W9" s="23"/>
       <c r="X9" s="24" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="Y9" s="24"/>
       <c r="Z9" s="24"/>
@@ -3516,10 +3540,10 @@
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C10" s="26"/>
       <c r="D10" s="26"/>
@@ -3527,7 +3551,7 @@
       <c r="F10" s="26"/>
       <c r="G10" s="26"/>
       <c r="H10" s="26" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="I10" s="26"/>
       <c r="J10" s="26"/>
@@ -3537,7 +3561,7 @@
       <c r="N10" s="26"/>
       <c r="O10" s="26"/>
       <c r="P10" s="26" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="Q10" s="26"/>
       <c r="R10" s="26"/>
@@ -3557,10 +3581,10 @@
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -3568,17 +3592,17 @@
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
       <c r="H11" s="13" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="I11" s="13"/>
       <c r="J11" s="13"/>
       <c r="K11" s="12" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="L11" s="12"/>
       <c r="M11" s="12"/>
       <c r="N11" s="13" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="O11" s="13"/>
       <c r="P11" s="13"/>
@@ -3600,232 +3624,232 @@
     </row>
     <row r="12" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="29" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B12" s="30" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D12" s="31"/>
       <c r="E12" s="32" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="G12" s="33"/>
       <c r="H12" s="30" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I12" s="33" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="J12" s="33"/>
       <c r="K12" s="30" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="L12" s="33" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M12" s="33"/>
       <c r="N12" s="30" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="O12" s="33" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="P12" s="33"/>
       <c r="Q12" s="30" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="R12" s="33" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="S12" s="33"/>
       <c r="T12" s="30" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="U12" s="33" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="V12" s="33"/>
       <c r="W12" s="30" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="X12" s="33" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="Y12" s="33"/>
       <c r="Z12" s="30" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="AA12" s="33" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="AB12" s="33"/>
       <c r="AC12" s="30" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="AD12" s="34" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="AE12" s="34"/>
     </row>
     <row r="13" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="29"/>
       <c r="B13" s="30" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D13" s="31"/>
       <c r="E13" s="32" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F13" s="33" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G13" s="33"/>
       <c r="H13" s="30" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="I13" s="33" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="J13" s="33"/>
       <c r="K13" s="30" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="L13" s="33" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="M13" s="33"/>
       <c r="N13" s="30" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="O13" s="33" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="P13" s="33"/>
       <c r="Q13" s="30" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="R13" s="33" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="S13" s="33"/>
       <c r="T13" s="30" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="U13" s="33" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="V13" s="33"/>
       <c r="W13" s="30" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="X13" s="33" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="Y13" s="33"/>
       <c r="Z13" s="30" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AA13" s="33" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="AB13" s="33"/>
       <c r="AC13" s="30" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="AD13" s="34" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="AE13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="29"/>
       <c r="B14" s="30" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D14" s="31"/>
       <c r="E14" s="32" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G14" s="33"/>
       <c r="H14" s="30" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="I14" s="33" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="J14" s="33"/>
       <c r="K14" s="30" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="L14" s="33" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="M14" s="33"/>
       <c r="N14" s="30" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="O14" s="33" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="P14" s="33"/>
       <c r="Q14" s="30" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="R14" s="33" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="S14" s="33"/>
       <c r="T14" s="30" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="U14" s="33" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="V14" s="33"/>
       <c r="W14" s="30" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="X14" s="33" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="Y14" s="33"/>
       <c r="Z14" s="30" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="AA14" s="33" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="AB14" s="33"/>
       <c r="AC14" s="30" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="AD14" s="34" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="AE14" s="34"/>
     </row>
     <row r="15" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="29"/>
       <c r="B15" s="35" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D15" s="31"/>
       <c r="E15" s="36"/>
@@ -3858,7 +3882,7 @@
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="37" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B16" s="37"/>
       <c r="C16" s="37"/>
@@ -3882,7 +3906,7 @@
       <c r="R16" s="38"/>
       <c r="S16" s="38"/>
       <c r="T16" s="39" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="U16" s="39"/>
       <c r="V16" s="39"/>
@@ -3902,9 +3926,11 @@
     </row>
     <row r="18" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="42" t="s">
-        <v>90</v>
-      </c>
-      <c r="B18" s="43"/>
+        <v>93</v>
+      </c>
+      <c r="B18" s="43" t="s">
+        <v>94</v>
+      </c>
       <c r="C18" s="43"/>
       <c r="D18" s="43"/>
       <c r="E18" s="43"/>
@@ -3941,7 +3967,7 @@
     </row>
     <row r="20" s="45" customFormat="true" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="44" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B20" s="44"/>
       <c r="C20" s="44"/>
@@ -3977,7 +4003,7 @@
     <row r="21" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="46" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B22" s="46"/>
       <c r="C22" s="46"/>
@@ -4012,7 +4038,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="47" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B23" s="47"/>
       <c r="C23" s="47"/>
@@ -4047,7 +4073,7 @@
     </row>
     <row r="24" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="48" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B24" s="48"/>
       <c r="C24" s="48"/>
@@ -4082,7 +4108,7 @@
     </row>
     <row r="25" s="45" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="49" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B25" s="49"/>
       <c r="C25" s="49"/>
@@ -4117,10 +4143,10 @@
     </row>
     <row r="26" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="50" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B26" s="51" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C26" s="51"/>
       <c r="D26" s="51"/>
@@ -4132,7 +4158,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="52" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B27" s="52"/>
       <c r="C27" s="52"/>
@@ -4167,7 +4193,7 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="48" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B28" s="48"/>
       <c r="C28" s="48"/>
@@ -4202,10 +4228,10 @@
     </row>
     <row r="29" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="53" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B29" s="51" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C29" s="51"/>
       <c r="D29" s="51"/>
@@ -4218,7 +4244,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="52" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B30" s="52"/>
       <c r="C30" s="52"/>
@@ -4253,7 +4279,7 @@
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="54" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B31" s="54"/>
       <c r="C31" s="54"/>
@@ -4273,13 +4299,15 @@
     </row>
     <row r="33" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="56" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B33" s="57" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C33" s="57"/>
-      <c r="D33" s="12"/>
+      <c r="D33" s="12" t="s">
+        <v>110</v>
+      </c>
       <c r="E33" s="12"/>
       <c r="F33" s="12"/>
       <c r="G33" s="12"/>
@@ -4308,7 +4336,7 @@
     <row r="35" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="40"/>
       <c r="B35" s="57" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C35" s="57"/>
       <c r="D35" s="58"/>
@@ -4323,7 +4351,7 @@
       <c r="M35" s="58"/>
       <c r="N35" s="58"/>
       <c r="O35" s="59" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="P35" s="59"/>
       <c r="Q35" s="59"/>
@@ -4349,7 +4377,7 @@
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="47" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B37" s="47"/>
       <c r="C37" s="47"/>
@@ -4412,7 +4440,7 @@
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="63" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B39" s="63"/>
       <c r="C39" s="63"/>
@@ -4429,7 +4457,7 @@
       <c r="N39" s="64"/>
       <c r="O39" s="64"/>
       <c r="P39" s="65" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="Q39" s="65"/>
       <c r="R39" s="65"/>
@@ -4450,7 +4478,7 @@
     <row r="40" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="41" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="46" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B41" s="46"/>
       <c r="C41" s="46"/>
@@ -4485,7 +4513,7 @@
     </row>
     <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="66" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B42" s="66"/>
       <c r="C42" s="66"/>
@@ -4503,7 +4531,7 @@
       <c r="O42" s="67"/>
       <c r="P42" s="68"/>
       <c r="Q42" s="69" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="R42" s="69"/>
       <c r="S42" s="69"/>
@@ -4555,7 +4583,7 @@
     </row>
     <row r="44" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="73" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B44" s="73"/>
       <c r="C44" s="73"/>
@@ -4589,7 +4617,9 @@
       <c r="AE44" s="73"/>
     </row>
     <row r="45" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="61"/>
+      <c r="A45" s="61" t="s">
+        <v>120</v>
+      </c>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
       <c r="D45" s="61"/>
@@ -4619,7 +4649,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="75" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B46" s="75"/>
       <c r="C46" s="75"/>
@@ -4635,7 +4665,7 @@
       <c r="M46" s="64"/>
       <c r="N46" s="64"/>
       <c r="O46" s="76" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="P46" s="76"/>
       <c r="Q46" s="76"/>
@@ -4656,7 +4686,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="77" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="B47" s="77"/>
       <c r="C47" s="77"/>
@@ -4691,7 +4721,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="78" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B48" s="78"/>
       <c r="C48" s="78"/>
@@ -4759,7 +4789,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="M50" s="79" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="N50" s="79"/>
       <c r="O50" s="79"/>
@@ -4782,7 +4812,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="80" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="O51" s="81"/>
       <c r="P51" s="81"/>
@@ -4824,7 +4854,7 @@
     </row>
     <row r="53" s="83" customFormat="true" ht="50.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="82" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="B53" s="82"/>
       <c r="C53" s="82"/>
@@ -4865,7 +4895,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="85" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="B56" s="86"/>
       <c r="C56" s="86"/>
@@ -4933,7 +4963,7 @@
     </row>
     <row r="58" customFormat="false" ht="409.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="88" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="B58" s="88"/>
       <c r="C58" s="88"/>
@@ -5628,7 +5658,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: handle formatting of date in JS
</commit_message>
<xml_diff>
--- a/resources/Pauschale_Reiseaufwandsentschaedigung.xlsx
+++ b/resources/Pauschale_Reiseaufwandsentschaedigung.xlsx
@@ -47,7 +47,7 @@
     <t xml:space="preserve">Geburtsdatum:</t>
   </si>
   <si>
-    <t xml:space="preserve">{d.birthDate:formatD('DDMMYY')}</t>
+    <t xml:space="preserve">{d.birthDate}</t>
   </si>
   <si>
     <t xml:space="preserve">Ausländische Sozialversicherungsnummer*:</t>
@@ -2261,9 +2261,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>30</xdr:col>
-      <xdr:colOff>110160</xdr:colOff>
+      <xdr:colOff>109800</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>105120</xdr:rowOff>
+      <xdr:rowOff>104760</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2277,7 +2277,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="7960320" y="185400"/>
-          <a:ext cx="2833200" cy="376920"/>
+          <a:ext cx="2832840" cy="376560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>